<commit_message>
Add vps_test_run2 and vps_test_run3 logs; address Oracle Client library errors and module import issues
</commit_message>
<xml_diff>
--- a/planilhas_cache/METAS SP.xlsx
+++ b/planilhas_cache/METAS SP.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Drives compartilhados\Off Trade\Campanhas e Metas\METAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E8FC689-3881-46FB-941E-C1BDE7A87CE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7E72D6F-B6B6-47EE-B991-2E61BB512F22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="META_VENDEDOR" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="92">
   <si>
     <t>RCA</t>
   </si>
@@ -306,6 +306,18 @@
   </si>
   <si>
     <t>PAULO MOREIRA - OFF TRADE</t>
+  </si>
+  <si>
+    <t>META FATURAMENTO CASTAS</t>
+  </si>
+  <si>
+    <t>PESO FATURAMENTO CASTAS</t>
+  </si>
+  <si>
+    <t>META FATURAMENTO ESSENZA + HOB</t>
+  </si>
+  <si>
+    <t>PESO FATURAMENTO ESSENZA + HOB</t>
   </si>
 </sst>
 </file>
@@ -2648,7 +2660,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4B0741B-ED62-42CC-8143-B374D33525D9}">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:Q3"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.33203125" style="12" bestFit="1" customWidth="1"/>
@@ -2663,10 +2675,13 @@
     <col min="10" max="11" width="24.77734375" style="11" customWidth="1"/>
     <col min="12" max="12" width="25.44140625" style="11" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="24.77734375" style="11" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.88671875" style="11"/>
+    <col min="14" max="14" width="26" style="11" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="25.5546875" style="11" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.44140625" style="11" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="8.88671875" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
         <v>55</v>
       </c>
@@ -2706,8 +2721,20 @@
       <c r="M1" s="20" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N1" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="O1" s="20" t="s">
+        <v>89</v>
+      </c>
+      <c r="P1" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="Q1" s="20" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
         <v>72</v>
       </c>
@@ -2746,6 +2773,55 @@
       </c>
       <c r="M2" s="18">
         <v>0</v>
+      </c>
+      <c r="N2" s="17"/>
+      <c r="O2" s="18"/>
+      <c r="P2" s="17"/>
+      <c r="Q2" s="18"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A3" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="C3" s="16">
+        <v>46204</v>
+      </c>
+      <c r="D3" s="17">
+        <v>5300000</v>
+      </c>
+      <c r="E3" s="18">
+        <v>0.7</v>
+      </c>
+      <c r="F3" s="19"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="17">
+        <v>3000000</v>
+      </c>
+      <c r="I3" s="18">
+        <v>0.05</v>
+      </c>
+      <c r="J3" s="17">
+        <v>300000</v>
+      </c>
+      <c r="K3" s="18">
+        <v>0.05</v>
+      </c>
+      <c r="L3" s="17"/>
+      <c r="M3" s="18"/>
+      <c r="N3" s="17">
+        <v>80000</v>
+      </c>
+      <c r="O3" s="18">
+        <v>0.1</v>
+      </c>
+      <c r="P3" s="17">
+        <v>35000</v>
+      </c>
+      <c r="Q3" s="18">
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add error logs for alerta_logistica_rj script due to missing 'bs4' module
- Created chunk_out.txt and chunk_out2.txt to capture error messages.
- Logged a ModuleNotFoundError indicating that the 'bs4' module is not installed.
</commit_message>
<xml_diff>
--- a/planilhas_cache/METAS SP.xlsx
+++ b/planilhas_cache/METAS SP.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Drives compartilhados\Off Trade\Campanhas e Metas\METAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7E72D6F-B6B6-47EE-B991-2E61BB512F22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3938EA9F-AB73-4BB6-A795-549C7CCE11B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="META_VENDEDOR" sheetId="1" r:id="rId1"/>
@@ -34,15 +34,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="92">
   <si>
     <t>RCA</t>
   </si>
@@ -324,12 +321,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="5">
+    <numFmt numFmtId="5" formatCode="&quot;R$&quot;\ #,##0;\-&quot;R$&quot;\ #,##0"/>
     <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #,##0.00"/>
+    <numFmt numFmtId="166" formatCode="0.00%;\-0.00%;0.00%"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -373,6 +372,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -441,7 +445,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -455,7 +459,6 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -492,8 +495,17 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="5" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -806,7 +818,6 @@
     <col min="13" max="13" width="28.21875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="28.6640625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="6.21875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="8.88671875" style="9"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
@@ -2216,7 +2227,7 @@
       <c r="B39" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C39" s="10" t="s">
+      <c r="C39" s="9" t="s">
         <v>70</v>
       </c>
       <c r="D39">
@@ -2233,7 +2244,7 @@
       <c r="B40" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C40" s="10" t="s">
+      <c r="C40" s="9" t="s">
         <v>61</v>
       </c>
       <c r="D40">
@@ -2250,7 +2261,7 @@
       <c r="B41" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C41" s="10" t="s">
+      <c r="C41" s="9" t="s">
         <v>62</v>
       </c>
       <c r="D41">
@@ -2267,7 +2278,7 @@
       <c r="B42" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C42" s="10" t="s">
+      <c r="C42" s="9" t="s">
         <v>63</v>
       </c>
       <c r="D42">
@@ -2284,7 +2295,7 @@
       <c r="B43" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C43" s="10" t="s">
+      <c r="C43" s="9" t="s">
         <v>64</v>
       </c>
       <c r="D43">
@@ -2301,7 +2312,7 @@
       <c r="B44" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C44" s="10" t="s">
+      <c r="C44" s="9" t="s">
         <v>65</v>
       </c>
       <c r="D44">
@@ -2318,7 +2329,7 @@
       <c r="B45" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C45" s="10" t="s">
+      <c r="C45" s="9" t="s">
         <v>66</v>
       </c>
       <c r="D45">
@@ -2335,7 +2346,7 @@
       <c r="B46" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C46" s="10" t="s">
+      <c r="C46" s="9" t="s">
         <v>67</v>
       </c>
       <c r="D46">
@@ -2352,7 +2363,7 @@
       <c r="B47" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C47" s="10" t="s">
+      <c r="C47" s="9" t="s">
         <v>68</v>
       </c>
       <c r="D47">
@@ -2369,7 +2380,7 @@
       <c r="B48" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C48" s="10" t="s">
+      <c r="C48" s="9" t="s">
         <v>69</v>
       </c>
       <c r="D48">
@@ -2386,7 +2397,7 @@
       <c r="B49" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C49" s="10" t="s">
+      <c r="C49" s="9" t="s">
         <v>81</v>
       </c>
       <c r="D49">
@@ -2403,7 +2414,7 @@
       <c r="B50" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C50" s="10" t="s">
+      <c r="C50" s="9" t="s">
         <v>82</v>
       </c>
       <c r="D50">
@@ -2420,7 +2431,7 @@
       <c r="B51" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C51" s="10" t="s">
+      <c r="C51" s="9" t="s">
         <v>83</v>
       </c>
       <c r="D51">
@@ -2437,7 +2448,7 @@
       <c r="B52" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C52" s="21" t="s">
+      <c r="C52" s="20" t="s">
         <v>84</v>
       </c>
       <c r="D52">
@@ -2454,7 +2465,7 @@
       <c r="B53" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C53" s="21" t="s">
+      <c r="C53" s="20" t="s">
         <v>85</v>
       </c>
       <c r="D53">
@@ -2471,7 +2482,7 @@
       <c r="B54" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C54" s="21" t="s">
+      <c r="C54" s="20" t="s">
         <v>86</v>
       </c>
       <c r="D54">
@@ -2488,7 +2499,7 @@
       <c r="B55" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C55" s="21" t="s">
+      <c r="C55" s="20" t="s">
         <v>87</v>
       </c>
       <c r="D55">
@@ -2499,7 +2510,7 @@
       </c>
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="C56" s="22"/>
+      <c r="C56" s="21"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C49:C56">
@@ -2512,145 +2523,243 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D508398-445A-42D1-9E23-A4409AC89A37}">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.33203125" style="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.33203125" style="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.33203125" style="11" customWidth="1"/>
-    <col min="4" max="4" width="18.33203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.77734375" style="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.5546875" style="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16" style="11" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="25.44140625" style="11" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.77734375" style="11" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="24.77734375" style="11" customWidth="1"/>
-    <col min="12" max="12" width="25.44140625" style="11" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="24.77734375" style="11" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.88671875" style="11"/>
+    <col min="1" max="1" width="11.33203125" style="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.33203125" style="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.33203125" style="10" customWidth="1"/>
+    <col min="4" max="4" width="18.33203125" style="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.77734375" style="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5546875" style="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16" style="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.44140625" style="10" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.77734375" style="10" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="24.77734375" style="10" customWidth="1"/>
+    <col min="12" max="12" width="25.44140625" style="10" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24.77734375" style="10" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="26" style="10" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="25.5546875" style="10" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="8.88671875" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
         <v>55</v>
       </c>
       <c r="B1" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="G1" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="20" t="s">
+      <c r="H1" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="I1" s="20" t="s">
+      <c r="I1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="J1" s="20" t="s">
+      <c r="J1" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="K1" s="20" t="s">
+      <c r="K1" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="20" t="s">
+      <c r="L1" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="M1" s="20" t="s">
+      <c r="M1" s="19" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A2" s="15" t="s">
+      <c r="N1" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="O1" s="19" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A2" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="C2" s="16">
-        <v>46174</v>
-      </c>
-      <c r="D2" s="17">
+      <c r="C2" s="15">
+        <v>46174</v>
+      </c>
+      <c r="D2" s="16">
         <v>1700000</v>
       </c>
-      <c r="E2" s="18">
+      <c r="E2" s="17">
         <v>0.4</v>
       </c>
-      <c r="F2" s="19">
+      <c r="F2" s="18">
         <v>130</v>
       </c>
-      <c r="G2" s="18">
+      <c r="G2" s="17">
         <v>0.25</v>
       </c>
-      <c r="H2" s="17">
+      <c r="H2" s="16">
         <v>1000000</v>
       </c>
-      <c r="I2" s="18">
+      <c r="I2" s="17">
         <v>0.1</v>
       </c>
-      <c r="J2" s="17">
+      <c r="J2" s="16">
         <v>20000</v>
       </c>
-      <c r="K2" s="18">
+      <c r="K2" s="17">
         <v>0.05</v>
       </c>
-      <c r="L2" s="17">
+      <c r="L2" s="16">
         <v>5000</v>
       </c>
-      <c r="M2" s="18">
+      <c r="M2" s="17">
         <v>0.2</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A3" s="15" t="s">
+      <c r="N2" s="18"/>
+      <c r="O2" s="18"/>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A3" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="C3" s="16">
-        <v>46174</v>
-      </c>
-      <c r="D3" s="17">
+      <c r="C3" s="15">
+        <v>46174</v>
+      </c>
+      <c r="D3" s="16">
         <v>1600000</v>
       </c>
-      <c r="E3" s="18">
+      <c r="E3" s="17">
         <v>0.4</v>
       </c>
-      <c r="F3" s="19">
+      <c r="F3" s="18">
         <v>90</v>
       </c>
-      <c r="G3" s="18">
+      <c r="G3" s="17">
         <v>0.25</v>
       </c>
-      <c r="H3" s="17">
+      <c r="H3" s="16">
         <v>1000000</v>
       </c>
-      <c r="I3" s="18">
+      <c r="I3" s="17">
         <v>0.1</v>
       </c>
-      <c r="J3" s="17">
+      <c r="J3" s="16">
         <v>20000</v>
       </c>
-      <c r="K3" s="18">
+      <c r="K3" s="17">
         <v>0.05</v>
       </c>
-      <c r="L3" s="17">
+      <c r="L3" s="16">
         <v>2000</v>
       </c>
-      <c r="M3" s="18">
+      <c r="M3" s="17">
         <v>0.2</v>
+      </c>
+      <c r="N3" s="18"/>
+      <c r="O3" s="18"/>
+    </row>
+    <row r="4" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A4" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="C4" s="15">
+        <v>46204</v>
+      </c>
+      <c r="D4" s="22">
+        <v>2200000</v>
+      </c>
+      <c r="E4" s="23">
+        <v>0.7</v>
+      </c>
+      <c r="F4" s="18"/>
+      <c r="G4" s="18"/>
+      <c r="H4" s="22">
+        <v>1000000</v>
+      </c>
+      <c r="I4" s="23">
+        <v>0.1</v>
+      </c>
+      <c r="J4" s="22">
+        <v>100000</v>
+      </c>
+      <c r="K4" s="23">
+        <v>0.05</v>
+      </c>
+      <c r="L4" s="22">
+        <v>10000</v>
+      </c>
+      <c r="M4" s="23">
+        <v>0.05</v>
+      </c>
+      <c r="N4" s="24">
+        <v>20000</v>
+      </c>
+      <c r="O4" s="23">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A5" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="C5" s="15">
+        <v>46204</v>
+      </c>
+      <c r="D5" s="22">
+        <v>1800000</v>
+      </c>
+      <c r="E5" s="23">
+        <v>0.7</v>
+      </c>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="22">
+        <v>1000000</v>
+      </c>
+      <c r="I5" s="23">
+        <v>0.1</v>
+      </c>
+      <c r="J5" s="22">
+        <v>100000</v>
+      </c>
+      <c r="K5" s="23">
+        <v>0.05</v>
+      </c>
+      <c r="L5" s="22">
+        <v>10000</v>
+      </c>
+      <c r="M5" s="23">
+        <v>0.05</v>
+      </c>
+      <c r="N5" s="24">
+        <v>20000</v>
+      </c>
+      <c r="O5" s="23">
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>
@@ -2663,164 +2772,165 @@
   <dimension ref="A1:Q3"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.33203125" style="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.33203125" style="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.33203125" style="11" customWidth="1"/>
-    <col min="4" max="4" width="18.33203125" style="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.77734375" style="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.5546875" style="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16" style="11" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="25.44140625" style="11" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.77734375" style="11" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="24.77734375" style="11" customWidth="1"/>
-    <col min="12" max="12" width="25.44140625" style="11" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="24.77734375" style="11" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="26" style="11" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="25.5546875" style="11" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.44140625" style="11" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="8.88671875" style="11"/>
+    <col min="1" max="1" width="11.33203125" style="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.33203125" style="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.33203125" style="10" customWidth="1"/>
+    <col min="4" max="4" width="18.33203125" style="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.77734375" style="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5546875" style="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16" style="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.44140625" style="10" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.77734375" style="10" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="24.77734375" style="10" customWidth="1"/>
+    <col min="12" max="12" width="25.44140625" style="10" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24.77734375" style="10" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="26" style="10" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="25.5546875" style="10" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="31.5546875" style="10" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="31.109375" style="10" bestFit="1" customWidth="1"/>
+    <col min="18" max="16384" width="8.88671875" style="10"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="G1" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="20" t="s">
+      <c r="H1" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="I1" s="20" t="s">
+      <c r="I1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="J1" s="20" t="s">
+      <c r="J1" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="K1" s="20" t="s">
+      <c r="K1" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="20" t="s">
+      <c r="L1" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="M1" s="20" t="s">
+      <c r="M1" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="N1" s="20" t="s">
+      <c r="N1" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="O1" s="20" t="s">
+      <c r="O1" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="P1" s="20" t="s">
+      <c r="P1" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="Q1" s="20" t="s">
+      <c r="Q1" s="19" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="C2" s="16">
-        <v>46174</v>
-      </c>
-      <c r="D2" s="17">
+      <c r="C2" s="15">
+        <v>46174</v>
+      </c>
+      <c r="D2" s="16">
         <v>4100000</v>
       </c>
-      <c r="E2" s="18">
+      <c r="E2" s="17">
         <v>0.8</v>
       </c>
-      <c r="F2" s="19">
+      <c r="F2" s="18">
         <v>380</v>
       </c>
-      <c r="G2" s="18">
+      <c r="G2" s="17">
         <v>0.1</v>
       </c>
-      <c r="H2" s="17">
+      <c r="H2" s="16">
         <v>3100000</v>
       </c>
-      <c r="I2" s="18">
+      <c r="I2" s="17">
         <v>0.05</v>
       </c>
-      <c r="J2" s="17">
+      <c r="J2" s="16">
         <v>100000</v>
       </c>
-      <c r="K2" s="18">
+      <c r="K2" s="17">
         <v>0.05</v>
       </c>
-      <c r="L2" s="17">
+      <c r="L2" s="16">
         <v>20000</v>
       </c>
-      <c r="M2" s="18">
+      <c r="M2" s="17">
         <v>0</v>
       </c>
-      <c r="N2" s="17"/>
-      <c r="O2" s="18"/>
-      <c r="P2" s="17"/>
-      <c r="Q2" s="18"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="17"/>
+      <c r="P2" s="16"/>
+      <c r="Q2" s="17"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="C3" s="16">
+      <c r="C3" s="15">
         <v>46204</v>
       </c>
-      <c r="D3" s="17">
+      <c r="D3" s="16">
         <v>5300000</v>
       </c>
-      <c r="E3" s="18">
+      <c r="E3" s="17">
         <v>0.7</v>
       </c>
-      <c r="F3" s="19"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="17">
+      <c r="F3" s="18"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="16">
         <v>3000000</v>
       </c>
-      <c r="I3" s="18">
+      <c r="I3" s="17">
         <v>0.05</v>
       </c>
-      <c r="J3" s="17">
+      <c r="J3" s="16">
         <v>300000</v>
       </c>
-      <c r="K3" s="18">
+      <c r="K3" s="17">
         <v>0.05</v>
       </c>
-      <c r="L3" s="17"/>
-      <c r="M3" s="18"/>
-      <c r="N3" s="17">
+      <c r="L3" s="16"/>
+      <c r="M3" s="17"/>
+      <c r="N3" s="16">
         <v>80000</v>
       </c>
-      <c r="O3" s="18">
+      <c r="O3" s="17">
         <v>0.1</v>
       </c>
-      <c r="P3" s="17">
+      <c r="P3" s="16">
         <v>35000</v>
       </c>
-      <c r="Q3" s="18">
+      <c r="Q3" s="17">
         <v>0.1</v>
       </c>
     </row>

</xml_diff>